<commit_message>
Enviar por correo: lista por dpto con botón Enviar (Gmail/mailto), PDF individual y mensaje con formato
</commit_message>
<xml_diff>
--- a/plantilla-ejemplo.xlsx
+++ b/plantilla-ejemplo.xlsx
@@ -457,7 +457,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">  Departamentos: un renglón por departamento (unidad y propietario).</v>
+        <v xml:space="preserve">  Departamentos: un renglón por departamento (unidad, propietario y correo; si hay varios correos, sepáralos con coma).</v>
       </c>
     </row>
     <row r="11">
@@ -504,7 +504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -645,73 +645,84 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EMPRESA_AGUA</v>
+        <v>CORREO_NOMBRE_EDIFICIO</v>
       </c>
       <c r="B13" t="str">
-        <v>Sedapal</v>
+        <v/>
       </c>
       <c r="C13" t="str">
-        <v>Empresa de agua (ej. Sedapal)</v>
+        <v>Opcional: nombre en el encabezado del correo (vacío = "Edificio" + nombre del edificio)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>EMPRESA_LUZ</v>
+        <v>EMPRESA_AGUA</v>
       </c>
       <c r="B14" t="str">
-        <v>Luz del Sur</v>
+        <v>Sedapal</v>
       </c>
       <c r="C14" t="str">
-        <v>Empresa de luz (ej. Luz del Sur)</v>
+        <v>Empresa de agua (ej. Sedapal)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>NUM_DPTOS</v>
-      </c>
-      <c r="B15">
-        <v>10</v>
+        <v>EMPRESA_LUZ</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Luz del Sur</v>
       </c>
       <c r="C15" t="str">
-        <v>Número de departamentos entre los que se dividen los gastos (vacío = los de la pestaña Departamentos)</v>
+        <v>Empresa de luz (ej. Luz del Sur)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>DIA_VENCIMIENTO</v>
+        <v>NUM_DPTOS</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C16" t="str">
-        <v>Día del mes siguiente en que vence el recibo (ej. 5)</v>
+        <v>Número de departamentos entre los que se dividen los gastos (vacío = los de la pestaña Departamentos)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SALDO_INICIAL_FONDO</v>
+        <v>DIA_VENCIMIENTO</v>
       </c>
       <c r="B17">
-        <v>4097.67</v>
+        <v>5</v>
       </c>
       <c r="C17" t="str">
-        <v>Saldo del fondo de contingencia antes del primer mes registrado</v>
+        <v>Día del mes siguiente en que vence el recibo (ej. 5)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>SALDO_INICIAL_FONDO</v>
+      </c>
+      <c r="B18">
+        <v>4097.67</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Saldo del fondo de contingencia antes del primer mes registrado</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>LOGO_BASE64</v>
       </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
         <v>Opcional: logo como texto base64 (más fácil: súbelo en la página y se guarda en la pestaña Logo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -738,7 +749,7 @@
         <v>Celular / WhatsApp</v>
       </c>
       <c r="D1" t="str">
-        <v>Correo</v>
+        <v>Correo(s) del propietario (varios: separar con coma)</v>
       </c>
       <c r="E1" t="str">
         <v>Notas</v>
@@ -755,7 +766,7 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>dpto101@ejemplo.com</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -772,7 +783,7 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>dpto102@ejemplo.com, inquilino102@ejemplo.com</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -789,7 +800,7 @@
         <v/>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>dpto201@ejemplo.com</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -806,7 +817,7 @@
         <v/>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>dpto202@ejemplo.com</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -823,7 +834,7 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>dpto301@ejemplo.com</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -840,7 +851,7 @@
         <v/>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>dpto302@ejemplo.com</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -857,7 +868,7 @@
         <v/>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>dpto401@ejemplo.com</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -874,7 +885,7 @@
         <v/>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>dpto402@ejemplo.com</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -891,7 +902,7 @@
         <v/>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>dpto501@ejemplo.com</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -908,7 +919,7 @@
         <v/>
       </c>
       <c r="D11" t="str">
-        <v/>
+        <v>dpto502@ejemplo.com</v>
       </c>
       <c r="E11" t="str">
         <v/>

</xml_diff>

<commit_message>
Sin ZIP: PDF por dpto + Excel actualizado; Google Drive con un botón (conectar/desconectar, subida con link público); correo con VER RECIBO y WhatsApp; guía PDF
</commit_message>
<xml_diff>
--- a/plantilla-ejemplo.xlsx
+++ b/plantilla-ejemplo.xlsx
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120.83203125" customWidth="1" min="1" max="1"/>
@@ -1411,77 +1411,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Sube las fotos y pulsa "Generar recibos": se descarga un ZIP con los PDF y este Excel ACTUALIZADO, con la pestaña "Mes a facturar" lista para el mes siguiente.</t>
+          <t>4. Sube las fotos y pulsa "Generar recibos": aparece la lista de departamentos con su PDF, y los botones para enviar por correo y WhatsApp.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Descarga también el Excel ACTUALIZADO (botón "Descargar Excel actualizado"): ya trae la pestaña "Mes a facturar" lista para el mes siguiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Guarda el Excel nuevo en lugar de este.</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Pestañas:</t>
-        </is>
-      </c>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Mes a facturar: lo único que se llena cada mes.</t>
+          <t>Pestañas:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Config: datos del edificio (presidente, tesorero, banco, cuenta, CCI, día de vencimiento...). Cambia solo la columna B.</t>
+          <t xml:space="preserve">  Mes a facturar: lo único que se llena cada mes.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Departamentos: un renglón por departamento (unidad, propietario y correo; si hay varios correos, sepáralos con coma).</t>
+          <t xml:space="preserve">  Config: datos del edificio (presidente, tesorero, banco, cuenta, CCI, titular, WhatsApp de constancias, día de vencimiento...). Cambia solo la columna B.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Lecturas, Servicios, Gastos, Ajustes, Fondo: historial de los meses ya generados (la página los llena sola; no hace falta tocarlos).</t>
+          <t xml:space="preserve">  Departamentos: un renglón por departamento (unidad, propietario, celular/WhatsApp de 9 dígitos y correo; si hay varios correos, sepáralos con coma).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipos de gasto: FIJO, EXTRA (no se repite), FONDO (aporte al fondo de contingencia), LUZ (= recibo de luz), AGUA_COMUN (se calcula solo).</t>
+          <t xml:space="preserve">  Lecturas, Servicios, Gastos, Ajustes, Fondo: historial de los meses ya generados (la página los llena sola; no hace falta tocarlos).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Tipos de gasto: FIJO, EXTRA (no se repite), FONDO (aporte al fondo de contingencia), LUZ (= recibo de luz), AGUA_COMUN (se calcula solo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Logo: lo llena la página si subes el logo. No la edites.</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Cálculo: cada gasto se divide entre el número de dptos; el agua de cada dpto = consumo × (monto del recibo de agua ÷ m³ facturados);</t>
-        </is>
-      </c>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>Cálculo: cada gasto se divide entre el número de dptos; el agua de cada dpto = consumo × (monto del recibo de agua ÷ m³ facturados);</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>el agua común = (m³ del recibo − m³ de los dptos) × precio; el céntimo de redondeo del agua va al dpto de mayor consumo.</t>
         </is>
@@ -1498,7 +1505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.83203125" customWidth="1" min="1" max="1"/>
@@ -1696,124 +1703,158 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>NOTA_PAGO</t>
+          <t>TITULAR_CUENTA</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Por favor, envíe su comprobante de pago al tesorero vía WhatsApp indicando su número de departamento.</t>
+          <t>Luis Gómez Ejemplo</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Nota que sale junto a los datos de pago</t>
+          <t>Titular de la cuenta (nombre completo; sale en el correo y en el WhatsApp)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>CORREO_NOMBRE_EDIFICIO</t>
+          <t>WHATSAPP_CONSTANCIA</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Edificio Ejemplo</t>
+          <t>999 000 222</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Opcional: nombre en el encabezado del correo (vacío = "Edificio" + nombre del edificio)</t>
+          <t>WhatsApp donde se envía la constancia de pago (vacío = celular del tesorero)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>EMPRESA_AGUA</t>
+          <t>NOTA_PAGO</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Sedapal</t>
+          <t>Por favor, envíe su comprobante de pago al tesorero vía WhatsApp indicando su número de departamento.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Empresa de agua (ej. Sedapal)</t>
+          <t>Nota que sale junto a los datos de pago</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>EMPRESA_LUZ</t>
+          <t>CORREO_NOMBRE_EDIFICIO</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Luz del Sur</t>
+          <t>Edificio Ejemplo</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Empresa de luz (ej. Luz del Sur)</t>
+          <t>Opcional: nombre en el encabezado del correo (vacío = "Edificio" + nombre del edificio)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>NUM_DPTOS</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>10</v>
+          <t>EMPRESA_AGUA</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Sedapal</t>
+        </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Número de departamentos entre los que se dividen los gastos (vacío = los de la pestaña Departamentos)</t>
+          <t>Empresa de agua (ej. Sedapal)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>DIA_VENCIMIENTO</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>5</v>
+          <t>EMPRESA_LUZ</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Luz del Sur</t>
+        </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Día del mes siguiente en que vence el recibo (ej. 5)</t>
+          <t>Empresa de luz (ej. Luz del Sur)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>SALDO_INICIAL_FONDO</t>
+          <t>NUM_DPTOS</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>4097.67</v>
+        <v>10</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Saldo del fondo de contingencia antes del primer mes registrado</t>
+          <t>Número de departamentos entre los que se dividen los gastos (vacío = los de la pestaña Departamentos)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>DIA_VENCIMIENTO</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Día del mes siguiente en que vence el recibo (ej. 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>SALDO_INICIAL_FONDO</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>4097.67</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Saldo del fondo de contingencia antes del primer mes registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>LOGO_BASE64</t>
         </is>
       </c>
-      <c r="B19" s="4" t="str"/>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="B21" s="4" t="str"/>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Opcional: logo como texto base64 (más fácil: súbelo en la página y se guarda en la pestaña Logo)</t>
         </is>
@@ -1939,11 +1980,7 @@
           <t>Lucía Sample</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>999001202</t>
-        </is>
-      </c>
+      <c r="C5" s="4" t="str"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>dpto202@ejemplo.com</t>
@@ -2002,11 +2039,7 @@
           <t>Diego Ensayo</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>999001401</t>
-        </is>
-      </c>
+      <c r="C8" s="4" t="str"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
           <t>dpto401@ejemplo.com</t>

</xml_diff>